<commit_message>
Corregido un error en el filtrador, el cual no detectaba técnicas y subtécnicas SIN ningún DS o DC, y las declaraba como ONLY NETWORK DETECTION
</commit_message>
<xml_diff>
--- a/Obtención_Técnicas_MOBILE/TechniquesTacticsMitre/TechniquesTactics_v17.xlsx
+++ b/Obtención_Técnicas_MOBILE/TechniquesTacticsMitre/TechniquesTactics_v17.xlsx
@@ -1134,7 +1134,7 @@
         <v>6</v>
       </c>
       <c r="H3" s="76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1159,7 +1159,7 @@
         <v>8</v>
       </c>
       <c r="H4" s="77" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" thickBot="1">
@@ -1184,7 +1184,7 @@
         <v>4</v>
       </c>
       <c r="H5" s="78" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" thickBot="1"/>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="I12" s="97" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="K12" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="K14" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="K16" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2766,7 @@
       </c>
       <c r="K20" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="K35" s="62" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="K36" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="K39" s="62" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="K40" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3872,7 @@
       </c>
       <c r="K42" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="K45" s="62" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="K62" s="64" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       </c>
       <c r="K69" s="62" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -7410,7 +7410,7 @@
       </c>
       <c r="J3" s="70" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -7833,7 +7833,7 @@
       </c>
       <c r="J12" s="72" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -8162,7 +8162,7 @@
       </c>
       <c r="J19" s="70" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -8209,7 +8209,7 @@
       </c>
       <c r="J20" s="72" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -8585,7 +8585,7 @@
       </c>
       <c r="J28" s="72" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -8632,7 +8632,7 @@
       </c>
       <c r="J29" s="70" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -9431,7 +9431,7 @@
       </c>
       <c r="J46" s="72" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>

</xml_diff>